<commit_message>
Resuming work on four cells concept.
</commit_message>
<xml_diff>
--- a/bridgeCalc.xlsx
+++ b/bridgeCalc.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="28125"/>
   <workbookPr autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="-34720" yWindow="1520" windowWidth="30280" windowHeight="17960"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16060" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="fourCellsChart" sheetId="8" r:id="rId1"/>
@@ -113,10 +113,10 @@
     <t>In</t>
   </si>
   <si>
-    <t>Samle</t>
+    <t>Rate</t>
   </si>
   <si>
-    <t>Rate</t>
+    <t>Sample</t>
   </si>
 </sst>
 </file>
@@ -1513,11 +1513,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="-2114874280"/>
-        <c:axId val="-2114905800"/>
+        <c:axId val="2103905384"/>
+        <c:axId val="2103908440"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="-2114874280"/>
+        <c:axId val="2103905384"/>
         <c:scaling>
           <c:logBase val="10.0"/>
           <c:orientation val="minMax"/>
@@ -1532,14 +1532,14 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="cross"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2114905800"/>
+        <c:crossAx val="2103908440"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="10.0"/>
         <c:minorUnit val="10.0"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-2114905800"/>
+        <c:axId val="2103908440"/>
         <c:scaling>
           <c:logBase val="10.0"/>
           <c:orientation val="minMax"/>
@@ -1554,7 +1554,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="cross"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="-2114874280"/>
+        <c:crossAx val="2103905384"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="10.0"/>
@@ -1585,7 +1585,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="9211623" cy="5616039"/>
+    <xdr:ext cx="9214662" cy="5624286"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1"/>
@@ -1921,7 +1921,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1974,7 +1974,7 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>3</v>
@@ -2006,7 +2006,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>

</xml_diff>